<commit_message>
docs: sync October 18 P0 verification and issue tracker
Update all 49 P0 progress rows and record menu gaps and requirement deviations. Results remain tied to reviewed commit 08a27c1; newer task 17b and 27 changes require retesting.

Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/docs/04-开发任务/CRM系统功能评估与进度跟踪表-1018.xlsx
+++ b/docs/04-开发任务/CRM系统功能评估与进度跟踪表-1018.xlsx
@@ -3494,7 +3494,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -3659,6 +3659,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="top"/>
+    </xf>
+    <xf xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="50">
@@ -4281,8 +4287,8 @@
     <col min="4" max="4" width="33.1333333333333" style="7" customWidth="1"/>
     <col min="5" max="5" width="83.6666666666667" style="7" customWidth="1"/>
     <col min="6" max="6" width="33.2166666666667" style="8" customWidth="1"/>
-    <col min="7" max="7" width="22.375" style="8" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="25" style="9" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="22.375" style="8" customWidth="1"/>
+    <col min="8" max="8" width="25" style="9" customWidth="1"/>
     <col min="9" max="9" width="35.9916666666667" style="7" customWidth="1"/>
     <col min="10" max="16384" width="9" style="7"/>
   </cols>
@@ -4382,7 +4388,12 @@
       <c r="G7" s="26">
         <v>46317</v>
       </c>
-      <c r="H7" s="22"/>
+      <c r="H7" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+邀请链接可用。未单独展示邀请码，管理员入口报错。</t>
+        </is>
+      </c>
       <c r="I7" s="7" t="str">
         <f>_xlfn.DISPIMG("ID_983306F5483D461FA3FFA10D90D826B7",1)</f>
         <v>=DISPIMG("ID_983306F5483D461FA3FFA10D90D826B7",1)</v>
@@ -4405,7 +4416,12 @@
       <c r="G8" s="48">
         <v>46316</v>
       </c>
-      <c r="H8" s="33"/>
+      <c r="H8" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+缺手填邀请码入口。通讯及社媒信息仍必填，与选填要求不符。</t>
+        </is>
+      </c>
       <c r="I8" s="7" t="str">
         <f>_xlfn.DISPIMG("ID_6406BE1B533C4808A9200C237918C668",1)</f>
         <v>=DISPIMG("ID_6406BE1B533C4808A9200C237918C668",1)</v>
@@ -4428,7 +4444,12 @@
       <c r="G9" s="26">
         <v>46317</v>
       </c>
-      <c r="H9" s="22"/>
+      <c r="H9" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 本地通过
+重复及大小写邮箱注册被拦截，已有账号可转登录。</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="60.75" customHeight="1" spans="2:9">
       <c r="B10" s="49" t="s">
@@ -4447,7 +4468,12 @@
       <c r="G10" s="32">
         <v>46317</v>
       </c>
-      <c r="H10" s="33"/>
+      <c r="H10" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 本地通过
+登录、停用拦截、密码重置通过。真实邮件投递待联调。</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="76.5" customHeight="1" spans="2:9">
       <c r="B11" s="47" t="s">
@@ -4466,7 +4492,12 @@
       <c r="G11" s="51">
         <v>46317</v>
       </c>
-      <c r="H11" s="22"/>
+      <c r="H11" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+已生成固定ID及待审核状态。ID多了KOL-前缀，需对齐。</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="54" customHeight="1" spans="2:9">
       <c r="B12" s="49" t="s">
@@ -4485,7 +4516,12 @@
       <c r="G12" s="32">
         <v>46318</v>
       </c>
-      <c r="H12" s="33"/>
+      <c r="H12" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 本地通过
+本人列表、名称筛选、精准认领、分页及越权拦截通过。</t>
+        </is>
+      </c>
       <c r="I12" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_EB10BD3009F54C148E61329E6E2F42D1",1)</f>
         <v>=DISPIMG("ID_EB10BD3009F54C148E61329E6E2F42D1",1)</v>
@@ -4510,7 +4546,12 @@
       <c r="G13" s="26">
         <v>46318</v>
       </c>
-      <c r="H13" s="22"/>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+有列表、编辑、启停和清理配置。缺预付及微店商品清理。</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="99" customHeight="1" spans="2:9">
       <c r="B14" s="49" t="s">
@@ -4529,7 +4570,12 @@
       <c r="G14" s="32">
         <v>46318</v>
       </c>
-      <c r="H14" s="33"/>
+      <c r="H14" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+自动绑定、首次审核已有。普通编辑可改邮箱，还可回待审核。</t>
+        </is>
+      </c>
       <c r="I14" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_B536FF8803344A69B2DD73B7A3A5CCBD",1)</f>
         <v>=DISPIMG("ID_B536FF8803344A69B2DD73B7A3A5CCBD",1)</v>
@@ -4552,7 +4598,12 @@
       <c r="G15" s="26">
         <v>46318</v>
       </c>
-      <c r="H15" s="22"/>
+      <c r="H15" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+配置可保存。新平台及邀请码未正确用于跳转，版本记录可绕过。</t>
+        </is>
+      </c>
       <c r="I15" s="53" t="s">
         <v>36</v>
       </c>
@@ -4574,7 +4625,12 @@
       <c r="G16" s="26">
         <v>46326</v>
       </c>
-      <c r="H16" s="43"/>
+      <c r="H16" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+未见预付申请、附件、审批单及财务任务完整流程。</t>
+        </is>
+      </c>
       <c r="I16" s="53" t="s">
         <v>36</v>
       </c>
@@ -4596,7 +4652,12 @@
       <c r="G17" s="32">
         <v>46326</v>
       </c>
-      <c r="H17" s="43"/>
+      <c r="H17" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+未见预付打款登记、负余额及后续佣金抵扣。</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="76.5" customHeight="1" spans="2:9">
       <c r="B18" s="49" t="s">
@@ -4615,7 +4676,12 @@
       <c r="G18" s="32">
         <v>46318</v>
       </c>
-      <c r="H18" s="22"/>
+      <c r="H18" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+店铺列表可用。缺编码/渠道筛选、分页、容量及接口状态。</t>
+        </is>
+      </c>
       <c r="I18" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_A85F6535EBB34CD6824898C3C9414B00",1)</f>
         <v>=DISPIMG("ID_A85F6535EBB34CD6824898C3C9414B00",1)</v>
@@ -4638,7 +4704,12 @@
       <c r="G19" s="26">
         <v>46318</v>
       </c>
-      <c r="H19" s="22"/>
+      <c r="H19" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+可新建店铺。缺渠道、容量配置和刷新，当前还限制最多3店。</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="76.5" customHeight="1" spans="2:9">
       <c r="B20" s="49" t="s">
@@ -4657,7 +4728,12 @@
       <c r="G20" s="32">
         <v>46318</v>
       </c>
-      <c r="H20" s="22"/>
+      <c r="H20" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+后台有授权接口，店铺页缺去授权及分接口状态。未真实授权。</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="76.5" customHeight="1" spans="2:9">
       <c r="B21" s="49" t="s">
@@ -4676,7 +4752,12 @@
       <c r="G21" s="26">
         <v>46318</v>
       </c>
-      <c r="H21" s="22"/>
+      <c r="H21" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+未见源店标记、自动复制池及按容量自动分配。</t>
+        </is>
+      </c>
       <c r="I21" s="52"/>
     </row>
     <row r="22" ht="76.5" customHeight="1" spans="2:9">
@@ -4696,7 +4777,12 @@
       <c r="G22" s="32">
         <v>46318</v>
       </c>
-      <c r="H22" s="22"/>
+      <c r="H22" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+店铺启停通过。缺与源店、复制池、容量的联动维护。</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="76.5" customHeight="1" spans="2:9">
       <c r="B23" s="49" t="s">
@@ -4715,7 +4801,12 @@
       <c r="G23" s="26">
         <v>46318</v>
       </c>
-      <c r="H23" s="22"/>
+      <c r="H23" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+订单页有同步入口。店铺行缺单独拉订单、拉退款操作。</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="76.5" customHeight="1" spans="2:9">
       <c r="B24" s="49" t="s">
@@ -4734,7 +4825,12 @@
       <c r="G24" s="32">
         <v>46318</v>
       </c>
-      <c r="H24" s="22"/>
+      <c r="H24" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+可选达人及有效期。数量默认1000应为1，缺渠道容量选择。</t>
+        </is>
+      </c>
       <c r="I24" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_8EF2FE65629749CDA0CBBA7FB87FAD0F",1)</f>
         <v>=DISPIMG("ID_8EF2FE65629749CDA0CBBA7FB87FAD0F",1)</v>
@@ -4757,7 +4853,12 @@
       <c r="G25" s="26">
         <v>46318</v>
       </c>
-      <c r="H25" s="22"/>
+      <c r="H25" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+指定店铺生成Token报500。自动分配池及容量关联未接通。</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="76.5" customHeight="1" spans="2:9">
       <c r="B26" s="49" t="s">
@@ -4776,7 +4877,12 @@
       <c r="G26" s="32">
         <v>46318</v>
       </c>
-      <c r="H26" s="22"/>
+      <c r="H26" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+列表、筛选、分页及复制入口已有。接脚本实际复制尚未打通。</t>
+        </is>
+      </c>
       <c r="I26" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_6AB650E6942B44648C901EF99B3D4E81",1)</f>
         <v>=DISPIMG("ID_6AB650E6942B44648C901EF99B3D4E81",1)</v>
@@ -4799,7 +4905,12 @@
       <c r="G27" s="26">
         <v>46318</v>
       </c>
-      <c r="H27" s="22"/>
+      <c r="H27" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+有效、用尽、过期状态可显示。真实复制扣减未验证。</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="76.5" customHeight="1" spans="2:9">
       <c r="B28" s="49" t="s">
@@ -4818,7 +4929,12 @@
       <c r="G28" s="32">
         <v>46318</v>
       </c>
-      <c r="H28" s="22"/>
+      <c r="H28" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+未见脚本发起复制、微店建商品及关联复制任务的完整链路。</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="76.5" customHeight="1" spans="2:9">
       <c r="B29" s="49" t="s">
@@ -4837,7 +4953,12 @@
       <c r="G29" s="26">
         <v>46318</v>
       </c>
-      <c r="H29" s="22"/>
+      <c r="H29" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+缺商品复制任务列表、筛选、分页及详情入口。</t>
+        </is>
+      </c>
       <c r="I29" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_986DBC3A1513472083ED55D5C812516A",1)</f>
         <v>=DISPIMG("ID_986DBC3A1513472083ED55D5C812516A",1)</v>
@@ -4860,7 +4981,12 @@
       <c r="G30" s="32">
         <v>46318</v>
       </c>
-      <c r="H30" s="22"/>
+      <c r="H30" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+缺商品复制任务成功/失败汇总和错误明细。</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="76.5" customHeight="1" spans="2:9">
       <c r="B31" s="49" t="s">
@@ -4879,7 +5005,12 @@
       <c r="G31" s="26">
         <v>46318</v>
       </c>
-      <c r="H31" s="22"/>
+      <c r="H31" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+缺复制结果中新旧商品、店铺、链接及失败原因明细。</t>
+        </is>
+      </c>
       <c r="I31" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_5BDE962A4A3C4DAEBB2AF661B5C00836",1)</f>
         <v>=DISPIMG("ID_5BDE962A4A3C4DAEBB2AF661B5C00836",1)</v>
@@ -4902,7 +5033,12 @@
       <c r="G32" s="32">
         <v>46318</v>
       </c>
-      <c r="H32" s="22"/>
+      <c r="H32" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+上传推广表可建映射。菜单应归达人商品，商务总列表被拒绝。</t>
+        </is>
+      </c>
       <c r="I32" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_DE1661686E834CF0947C614B9807DD66",1)</f>
         <v>=DISPIMG("ID_DE1661686E834CF0947C614B9807DD66",1)</v>
@@ -4925,7 +5061,12 @@
       <c r="G33" s="48">
         <v>46326</v>
       </c>
-      <c r="H33" s="33"/>
+      <c r="H33" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+有禁用、转交及预约。缺本人离职及预约停用流程。</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="60.75" customHeight="1" spans="2:9">
       <c r="B34" s="49" t="s">
@@ -4944,7 +5085,12 @@
       <c r="G34" s="26">
         <v>46326</v>
       </c>
-      <c r="H34" s="22"/>
+      <c r="H34" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+立即转交、预约和撤销已验证。推广表商务名同步未实现。</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="54" customHeight="1" spans="2:9">
       <c r="B35" s="49" t="s">
@@ -4963,7 +5109,12 @@
       <c r="G35" s="48">
         <v>46326</v>
       </c>
-      <c r="H35" s="33"/>
+      <c r="H35" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 本地通过
+支付时商务归属保留，转交后历史订单及其退款不换商务。</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="54" customHeight="1" spans="2:9">
       <c r="B36" s="49" t="s">
@@ -4982,7 +5133,12 @@
       <c r="G36" s="26">
         <v>46326</v>
       </c>
-      <c r="H36" s="22"/>
+      <c r="H36" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+待更新及达人订单可见已验证。无主业绩、结算未闭环。</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="54" customHeight="1" spans="2:9">
       <c r="B37" s="49" t="s">
@@ -5001,7 +5157,12 @@
       <c r="G37" s="48">
         <v>46325</v>
       </c>
-      <c r="H37" s="33"/>
+      <c r="H37" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+收款审核按当前商务隔离。缺提现、预付待办的交接。</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="74" customHeight="1" spans="2:9">
       <c r="B38" s="47" t="s">
@@ -5020,7 +5181,12 @@
       <c r="G38" s="54" t="s">
         <v>106</v>
       </c>
-      <c r="H38" s="33"/>
+      <c r="H38" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+本机订单映射可用。真实成交未取样，跨达人合单及账务链路待核。</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="84" customHeight="1" spans="2:9">
       <c r="B39" s="49" t="s">
@@ -5039,7 +5205,12 @@
       <c r="G39" s="26">
         <v>46313</v>
       </c>
-      <c r="H39" s="22"/>
+      <c r="H39" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+订单基础状态及退款合计已有。缺退款类型/独立状态和统计验证。</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="75" customHeight="1" spans="2:9">
       <c r="B40" s="47" t="s">
@@ -5058,7 +5229,12 @@
       <c r="G40" s="54" t="s">
         <v>112</v>
       </c>
-      <c r="H40" s="33"/>
+      <c r="H40" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 待外部实测
+无真实微店授权和样本，订单、退款及计佣字段尚不能定论。</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="85" customHeight="1" spans="2:9">
       <c r="B41" s="49" t="s">
@@ -5077,7 +5253,12 @@
       <c r="G41" s="26">
         <v>46325</v>
       </c>
-      <c r="H41" s="22"/>
+      <c r="H41" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+有5分钟调度、分页和游标。真实退款状态及历史补偿待联调。</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="54" customHeight="1" spans="2:9">
       <c r="B42" s="49" t="s">
@@ -5096,7 +5277,12 @@
       <c r="G42" s="32">
         <v>46325</v>
       </c>
-      <c r="H42" s="33"/>
+      <c r="H42" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+表格导入、去重通过。CSV被拒绝，缺数据截止时间。</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="219" customHeight="1" spans="2:9">
       <c r="B43" s="49" t="s">
@@ -5115,7 +5301,12 @@
       <c r="G43" s="26">
         <v>46325</v>
       </c>
-      <c r="H43" s="22"/>
+      <c r="H43" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+有订单行和同步状态。缺订单号筛选、退款独立页及完整结算链路。</t>
+        </is>
+      </c>
       <c r="I43" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_CE7277A19C3549E0B2B4006DEDA8D43D",1)</f>
         <v>=DISPIMG("ID_CE7277A19C3549E0B2B4006DEDA8D43D",1)</v>
@@ -5138,7 +5329,12 @@
       <c r="G44" s="32">
         <v>46326</v>
       </c>
-      <c r="H44" s="33"/>
+      <c r="H44" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+匹配池、人工指定及原因校验已有。证据链展示不完整。</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="54" customHeight="1" spans="2:9">
       <c r="B45" s="49" t="s">
@@ -5157,7 +5353,12 @@
       <c r="G45" s="26">
         <v>46326</v>
       </c>
-      <c r="H45" s="22"/>
+      <c r="H45" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+人工改归属、原因留痕通过。缺已付差额及账务重算。</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="54" customHeight="1" spans="2:9">
       <c r="B46" s="47" t="s">
@@ -5176,7 +5377,12 @@
       <c r="G46" s="32">
         <v>46326</v>
       </c>
-      <c r="H46" s="33"/>
+      <c r="H46" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+仅能配置佣金比例，尚无按微店可提现金额计佣闭环。</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="131" customHeight="1" spans="2:9">
       <c r="B47" s="49" t="s">
@@ -5195,7 +5401,12 @@
       <c r="G47" s="26">
         <v>46326</v>
       </c>
-      <c r="H47" s="22"/>
+      <c r="H47" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+缺达人收入页、余额分层、收入流水及订单追溯。</t>
+        </is>
+      </c>
       <c r="I47" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_81CEA594730D4234AB8C0734B9C961B5",1)</f>
         <v>=DISPIMG("ID_81CEA594730D4234AB8C0734B9C961B5",1)</v>
@@ -5218,7 +5429,12 @@
       <c r="G48" s="32">
         <v>46326</v>
       </c>
-      <c r="H48" s="33"/>
+      <c r="H48" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+缺结算配置、200元门槛、冻结及占用/预付余额校验。</t>
+        </is>
+      </c>
       <c r="I48" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_5599563ED076454D876E46B483DB03A1",1)</f>
         <v>=DISPIMG("ID_5599563ED076454D876E46B483DB03A1",1)</v>
@@ -5241,7 +5457,12 @@
       <c r="G49" s="26">
         <v>46326</v>
       </c>
-      <c r="H49" s="22"/>
+      <c r="H49" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 部分实现
+收款账户维护及审核已有。缺每次提现填写及独立快照。</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="62" customHeight="1" spans="2:9">
       <c r="B50" s="49" t="s">
@@ -5260,7 +5481,12 @@
       <c r="G50" s="32">
         <v>46326</v>
       </c>
-      <c r="H50" s="33"/>
+      <c r="H50" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+收款账户审核不能替代提现审批，缺提现申请和财务任务。</t>
+        </is>
+      </c>
       <c r="I50" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_272A0461A4394375949F5C4798EB9C9E",1)</f>
         <v>=DISPIMG("ID_272A0461A4394375949F5C4798EB9C9E",1)</v>
@@ -5283,7 +5509,12 @@
       <c r="G51" s="26">
         <v>46326</v>
       </c>
-      <c r="H51" s="22"/>
+      <c r="H51" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+缺支付登记、支付凭证、幂等和佣金/预付记账。</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="58" customHeight="1" spans="2:9">
       <c r="B52" s="49" t="s">
@@ -5302,7 +5533,12 @@
       <c r="G52" s="32">
         <v>46326</v>
       </c>
-      <c r="H52" s="43"/>
+      <c r="H52" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+缺提现/预付申请记录及四类任务状态、付款明细。</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="60.75" spans="2:9">
       <c r="B53" s="49" t="s">
@@ -5318,8 +5554,14 @@
         <v>150</v>
       </c>
       <c r="F53" s="27"/>
-      <c r="G53" s="32">
+      <c r="G53" s="26">
         <v>46326</v>
+      </c>
+      <c r="H53" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+缺财务结算任务列表、筛选和审批/支付入口。</t>
+        </is>
       </c>
     </row>
     <row r="54" ht="56" customHeight="1" spans="2:9">
@@ -5336,6 +5578,15 @@
         <v>152</v>
       </c>
       <c r="F54" s="31"/>
+      <c r="G54" s="32">
+        <v>46326</v>
+      </c>
+      <c r="H54" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+缺结算任务详情、商品行占用、预付抵扣和支付凭证。</t>
+        </is>
+      </c>
       <c r="I54" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_4AE055A7E9A14962A0EB746E26F0624A",1)</f>
         <v>=DISPIMG("ID_4AE055A7E9A14962A0EB746E26F0624A",1)</v>
@@ -5355,6 +5606,15 @@
         <v>154</v>
       </c>
       <c r="F55" s="27"/>
+      <c r="G55" s="26">
+        <v>46326</v>
+      </c>
+      <c r="H55" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10/18 未实现
+缺结算明细、商品行账务流水和入账/付款分别记录。</t>
+        </is>
+      </c>
       <c r="I55" s="52" t="str">
         <f>_xlfn.DISPIMG("ID_298810721013485C89911230BB313995",1)</f>
         <v>=DISPIMG("ID_298810721013485C89911230BB313995",1)</v>

</xml_diff>

<commit_message>
docs: update P0 progress in 1018 tracker as of 2026-10-22
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/04-开发任务/CRM系统功能评估与进度跟踪表-1018.xlsx
+++ b/docs/04-开发任务/CRM系统功能评估与进度跟踪表-1018.xlsx
@@ -4390,8 +4390,8 @@
       </c>
       <c r="H7" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-邀请链接可用。未单独展示邀请码，管理员入口报错。</t>
+          <t xml:space="preserve">10/22 已实现
+邀请达人弹窗展示商务专属邀请码、注册链接及二维码。</t>
         </is>
       </c>
       <c r="I7" s="7" t="str">
@@ -4418,8 +4418,8 @@
       </c>
       <c r="H8" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-缺手填邀请码入口。通讯及社媒信息仍必填，与选填要求不符。</t>
+          <t xml:space="preserve">10/22 已实现
+链接注册自动填邀请码且只读；登录页注册可手填邀请码；联系方式与社媒为选填。</t>
         </is>
       </c>
       <c r="I8" s="7" t="str">
@@ -4446,7 +4446,7 @@
       </c>
       <c r="H9" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 本地通过
+          <t xml:space="preserve">10/22 已实现
 重复及大小写邮箱注册被拦截，已有账号可转登录。</t>
         </is>
       </c>
@@ -4470,8 +4470,8 @@
       </c>
       <c r="H10" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 本地通过
-登录、停用拦截、密码重置通过。真实邮件投递待联调。</t>
+          <t xml:space="preserve">10/22 已实现
+登录、停用拦截、密码重置通过。真实邮件投递待上线环境联调。</t>
         </is>
       </c>
     </row>
@@ -4494,8 +4494,8 @@
       </c>
       <c r="H11" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-已生成固定ID及待审核状态。ID多了KOL-前缀，需对齐。</t>
+          <t xml:space="preserve">10/22 已实现
+注册即生成固定编号，状态为待审核。编号按负责人决定带 KOL- 前缀（如 KOL-ASD001，ADR-023）。</t>
         </is>
       </c>
     </row>
@@ -4518,8 +4518,8 @@
       </c>
       <c r="H12" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 本地通过
-本人列表、名称筛选、精准认领、分页及越权拦截通过。</t>
+          <t xml:space="preserve">10/22 已实现
+商务只看本人达人，未绑定达人精准搜索后认领；按编号、名称、邮箱查询，分页。</t>
         </is>
       </c>
       <c r="I12" s="52" t="str">
@@ -4548,8 +4548,8 @@
       </c>
       <c r="H13" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-有列表、编辑、启停和清理配置。缺预付及微店商品清理。</t>
+          <t xml:space="preserve">10/22 部分实现
+列表字段、三种状态、编辑、审核、佣金、冻结、清理配置（自动/手动、删微店链接、清理明细）已有。预付金额属佣金结算，等微店结算数据确认（Q-1017-1/2）后开发。</t>
         </is>
       </c>
     </row>
@@ -4572,8 +4572,8 @@
       </c>
       <c r="H14" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-自动绑定、首次审核已有。普通编辑可改邮箱，还可回待审核。</t>
+          <t xml:space="preserve">10/22 已实现
+审核后不可再审，邮箱与编号只读；注册自动绑定商务，无有效商务显示待更新。</t>
         </is>
       </c>
       <c r="I14" s="52" t="str">
@@ -4600,8 +4600,8 @@
       </c>
       <c r="H15" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-配置可保存。新平台及邀请码未正确用于跳转，版本记录可绕过。</t>
+          <t xml:space="preserve">10/22 已实现
+佣金比例、平台及地址（可增删）、备注、版本与生效时间、修改记录。负责人确认不需要达人邀请码（10/21）。</t>
         </is>
       </c>
       <c r="I15" s="53" t="s">
@@ -4627,8 +4627,8 @@
       </c>
       <c r="H16" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-未见预付申请、附件、审批单及财务任务完整流程。</t>
+          <t xml:space="preserve">10/22 未实现
+达人列表预付入口显示「开发中」。预付流程由另一开发线在做（#104、#105 审查中，未合并）。</t>
         </is>
       </c>
       <c r="I16" s="53" t="s">
@@ -4654,8 +4654,8 @@
       </c>
       <c r="H17" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-未见预付打款登记、负余额及后续佣金抵扣。</t>
+          <t xml:space="preserve">10/22 未实现
+预付审批、付款登记与佣金抵扣由另一开发线在做（#104、#105 审查中，未合并）。</t>
         </is>
       </c>
     </row>
@@ -4678,8 +4678,8 @@
       </c>
       <c r="H18" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-店铺列表可用。缺编码/渠道筛选、分页、容量及接口状态。</t>
+          <t xml:space="preserve">10/22 已实现
+编码、名称、渠道筛选，分页，编码复制；源店铺、复制池、授权、接口状态、容量均已展示。</t>
         </is>
       </c>
       <c r="I18" s="52" t="str">
@@ -4706,8 +4706,8 @@
       </c>
       <c r="H19" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-可新建店铺。缺渠道、容量配置和刷新，当前还限制最多3店。</t>
+          <t xml:space="preserve">10/22 已实现
+新建/编辑含渠道、最大商品数（默认 20000）、容量刷新；公司店铺上限改为默认 20。</t>
         </is>
       </c>
     </row>
@@ -4730,8 +4730,8 @@
       </c>
       <c r="H20" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-后台有授权接口，店铺页缺去授权及分接口状态。未真实授权。</t>
+          <t xml:space="preserve">10/22 已实现（待微店实测）
+去授权、授权状态与过期时间、商品/订单/退款接口状态已有；真实微店授权待实测。</t>
         </is>
       </c>
     </row>
@@ -4754,8 +4754,8 @@
       </c>
       <c r="H21" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-未见源店标记、自动复制池及按容量自动分配。</t>
+          <t xml:space="preserve">10/22 已实现
+源店铺标记，复制池已加入/已退出/不参与；令牌按渠道剩余容量自动分配店铺。</t>
         </is>
       </c>
       <c r="I21" s="52"/>
@@ -4779,8 +4779,8 @@
       </c>
       <c r="H22" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-店铺启停通过。缺与源店、复制池、容量的联动维护。</t>
+          <t xml:space="preserve">10/22 已实现
+启停与源店铺、复制池、授权、容量联动判断能否作复制目标；行操作按负责人决定全部直接显示，不用「更多」（ADR-029）。</t>
         </is>
       </c>
     </row>
@@ -4803,8 +4803,8 @@
       </c>
       <c r="H23" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-订单页有同步入口。店铺行缺单独拉订单、拉退款操作。</t>
+          <t xml:space="preserve">10/22 已实现
+店铺行「拉订单」「拉退款」按所选店铺分别触发同步。</t>
         </is>
       </c>
     </row>
@@ -4827,8 +4827,8 @@
       </c>
       <c r="H24" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-可选达人及有效期。数量默认1000应为1，缺渠道容量选择。</t>
+          <t xml:space="preserve">10/22 已实现
+达人按名称/编码/邮箱搜索；目标渠道显示自动池剩余；数量默认 1，有效分钟默认 1440。</t>
         </is>
       </c>
       <c r="I24" s="52" t="str">
@@ -4855,8 +4855,8 @@
       </c>
       <c r="H25" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-指定店铺生成Token报500。自动分配池及容量关联未接通。</t>
+          <t xml:space="preserve">10/22 已实现
+可指定目标店铺或由自动池分配；数量超出剩余容量即拦截；指定店铺报 500 已修复。</t>
         </is>
       </c>
     </row>
@@ -4879,8 +4879,8 @@
       </c>
       <c r="H26" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-列表、筛选、分页及复制入口已有。接脚本实际复制尚未打通。</t>
+          <t xml:space="preserve">10/22 已实现（待微店实测）
+列表、筛选、分页、复制已有；表格脚本对接接口已完成，真实复制待微店授权实测。</t>
         </is>
       </c>
       <c r="I26" s="52" t="str">
@@ -4907,8 +4907,8 @@
       </c>
       <c r="H27" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-有效、用尽、过期状态可显示。真实复制扣减未验证。</t>
+          <t xml:space="preserve">10/22 已实现（待微店实测）
+已用/总量与有效、已用尽、已过期状态已有；真实复制扣减待实测。</t>
         </is>
       </c>
     </row>
@@ -4931,8 +4931,8 @@
       </c>
       <c r="H28" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-未见脚本发起复制、微店建商品及关联复制任务的完整链路。</t>
+          <t xml:space="preserve">10/22 已实现（待微店实测）
+表格脚本复制接口与商品任务关联已完成；真实微店建商品待 M0 实测。</t>
         </is>
       </c>
     </row>
@@ -4955,8 +4955,8 @@
       </c>
       <c r="H29" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-缺商品复制任务列表、筛选、分页及详情入口。</t>
+          <t xml:space="preserve">10/22 已实现
+商品任务列表按编号、渠道、状态查询，编号复制，重置、刷新、分页。</t>
         </is>
       </c>
       <c r="I29" s="52" t="str">
@@ -4983,8 +4983,8 @@
       </c>
       <c r="H30" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-缺商品复制任务成功/失败汇总和错误明细。</t>
+          <t xml:space="preserve">10/22 已实现
+展示总数、成功、失败及任务级错误；已完成任务中的失败项可见。</t>
         </is>
       </c>
     </row>
@@ -5007,8 +5007,8 @@
       </c>
       <c r="H31" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-缺复制结果中新旧商品、店铺、链接及失败原因明细。</t>
+          <t xml:space="preserve">10/22 已实现
+明细含来源/目标渠道、店铺、商户号、新旧商品 ID、新商品链接、状态与失败原因。</t>
         </is>
       </c>
       <c r="I31" s="52" t="str">
@@ -5035,8 +5035,8 @@
       </c>
       <c r="H32" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-上传推广表可建映射。菜单应归达人商品，商务总列表被拒绝。</t>
+          <t xml:space="preserve">10/22 已实现
+「达人管理—达人商品」含链接编码、主图、销量、支付金额、清理状态与详情，并衔接订单链路。</t>
         </is>
       </c>
       <c r="I32" s="52" t="str">
@@ -5063,8 +5063,8 @@
       </c>
       <c r="H33" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-有禁用、转交及预约。缺本人离职及预约停用流程。</t>
+          <t xml:space="preserve">10/22 已实现
+本人申请离职；管理员标记离职/停用，可预约；到期按继承商务转移达人并停用账号。</t>
         </is>
       </c>
     </row>
@@ -5087,8 +5087,8 @@
       </c>
       <c r="H34" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-立即转交、预约和撤销已验证。推广表商务名同步未实现。</t>
+          <t xml:space="preserve">10/22 已实现
+单个、批量、立即与预约转交已验证；推广表不入库，商务名同步不适用。</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5111,7 @@
       </c>
       <c r="H35" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 本地通过
+          <t xml:space="preserve">10/22 已实现
 支付时商务归属保留，转交后历史订单及其退款不换商务。</t>
         </is>
       </c>
@@ -5135,8 +5135,8 @@
       </c>
       <c r="H36" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-待更新及达人订单可见已验证。无主业绩、结算未闭环。</t>
+          <t xml:space="preserve">10/22 部分实现
+无商务期间订单的商务为空，即无主业绩；计入管理员的业绩统计随看板（P1），佣金结算未实现。</t>
         </is>
       </c>
     </row>
@@ -5159,8 +5159,8 @@
       </c>
       <c r="H37" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-收款审核按当前商务隔离。缺提现、预付待办的交接。</t>
+          <t xml:space="preserve">10/22 部分实现
+收款账户待审核随转交归新商务。提现、预付待办属佣金结算，等微店结算数据确认（Q-1017-1/2）后开发。</t>
         </is>
       </c>
     </row>
@@ -5183,8 +5183,8 @@
       </c>
       <c r="H38" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-本机订单映射可用。真实成交未取样，跨达人合单及账务链路待核。</t>
+          <t xml:space="preserve">10/22 待外部实测
+订单链路页已实现（任务→链接编码→订单→退款）；真实成交取样待微店授权；账务流水、提现占用显示「开发中」。</t>
         </is>
       </c>
     </row>
@@ -5207,8 +5207,8 @@
       </c>
       <c r="H39" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-订单基础状态及退款合计已有。缺退款类型/独立状态和统计验证。</t>
+          <t xml:space="preserve">10/22 已实现（待微店实测）
+订单状态、退款状态、退款类型分列记录和展示，退款中不计成功退款；真实状态取值待 M0 核实。</t>
         </is>
       </c>
     </row>
@@ -5231,7 +5231,7 @@
       </c>
       <c r="H40" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 待外部实测
+          <t xml:space="preserve">10/22 待外部实测
 无真实微店授权和样本，订单、退款及计佣字段尚不能定论。</t>
         </is>
       </c>
@@ -5255,8 +5255,8 @@
       </c>
       <c r="H41" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-有5分钟调度、分页和游标。真实退款状态及历史补偿待联调。</t>
+          <t xml:space="preserve">10/22 部分实现
+5 分钟调度、分页、游标；订单与退款分别同步，每笔退款单独保留。真实退款状态及历史补偿待联调。</t>
         </is>
       </c>
     </row>
@@ -5279,8 +5279,8 @@
       </c>
       <c r="H42" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-表格导入、去重通过。CSV被拒绝，缺数据截止时间。</t>
+          <t xml:space="preserve">10/22 已实现
+Excel、CSV 导入与去重；导入必填数据截止时间，同步监控显示最近截止时间。真实导出文件待实测。</t>
         </is>
       </c>
     </row>
@@ -5303,8 +5303,8 @@
       </c>
       <c r="H43" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-有订单行和同步状态。缺订单号筛选、退款独立页及完整结算链路。</t>
+          <t xml:space="preserve">10/22 已实现（结算部分除外）
+订单查询与详情、退款查询与详情、订单链路、同步监控与失败任务已有；账务流水、提现占用显示「开发中」。</t>
         </is>
       </c>
       <c r="I43" s="52" t="str">
@@ -5331,8 +5331,8 @@
       </c>
       <c r="H44" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-匹配池、人工指定及原因校验已有。证据链展示不完整。</t>
+          <t xml:space="preserve">10/22 已实现
+匹配池可查看依据：商品 ID、店铺、达人映射与生效期（覆盖支付时间高亮）、未匹配原因、处理记录。</t>
         </is>
       </c>
     </row>
@@ -5355,8 +5355,8 @@
       </c>
       <c r="H45" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-人工改归属、原因留痕通过。缺已付差额及账务重算。</t>
+          <t xml:space="preserve">10/22 部分实现
+人工改归属、前后值与原因留痕已有。已付佣金差额与账务重算属佣金结算，等微店结算数据确认（Q-1017-1/2）后开发。</t>
         </is>
       </c>
     </row>
@@ -5379,8 +5379,8 @@
       </c>
       <c r="H46" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-仅能配置佣金比例，尚无按微店可提现金额计佣闭环。</t>
+          <t xml:space="preserve">10/22 未实现
+属佣金结算，等微店结算数据确认（Q-1017-1/2）后开发。</t>
         </is>
       </c>
     </row>
@@ -5403,8 +5403,8 @@
       </c>
       <c r="H47" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-缺达人收入页、余额分层、收入流水及订单追溯。</t>
+          <t xml:space="preserve">10/22 未实现
+达人收入页、余额分层、收入流水属佣金结算，等微店结算数据确认（Q-1017-1/2）后开发。</t>
         </is>
       </c>
       <c r="I47" s="52" t="str">
@@ -5431,8 +5431,8 @@
       </c>
       <c r="H48" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-缺结算配置、200元门槛、冻结及占用/预付余额校验。</t>
+          <t xml:space="preserve">10/22 未实现
+结算配置、提现门槛与冻结规则属佣金结算，等微店结算数据确认（Q-1017-1/2）后开发。</t>
         </is>
       </c>
       <c r="I48" s="52" t="str">
@@ -5459,8 +5459,8 @@
       </c>
       <c r="H49" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 部分实现
-收款账户维护及审核已有。缺每次提现填写及独立快照。</t>
+          <t xml:space="preserve">10/22 部分实现
+收款账户维护及审核已有。每次提现填写及快照属佣金结算，等微店结算数据确认（Q-1017-1/2）后开发。</t>
         </is>
       </c>
     </row>
@@ -5483,8 +5483,8 @@
       </c>
       <c r="H50" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-收款账户审核不能替代提现审批，缺提现申请和财务任务。</t>
+          <t xml:space="preserve">10/22 未实现
+提现申请与审批属佣金结算，等微店结算数据确认（Q-1017-1/2）后开发。</t>
         </is>
       </c>
       <c r="I50" s="52" t="str">
@@ -5511,8 +5511,8 @@
       </c>
       <c r="H51" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-缺支付登记、支付凭证、幂等和佣金/预付记账。</t>
+          <t xml:space="preserve">10/22 未实现
+支付登记、凭证与记账属佣金结算，等微店结算数据确认（Q-1017-1/2）后开发。</t>
         </is>
       </c>
     </row>
@@ -5535,8 +5535,8 @@
       </c>
       <c r="H52" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-缺提现/预付申请记录及四类任务状态、付款明细。</t>
+          <t xml:space="preserve">10/22 未实现
+提现/预付申请记录属佣金结算，等微店结算数据确认（Q-1017-1/2）后开发。</t>
         </is>
       </c>
     </row>
@@ -5559,8 +5559,8 @@
       </c>
       <c r="H53" s="60" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-缺财务结算任务列表、筛选和审批/支付入口。</t>
+          <t xml:space="preserve">10/22 未实现
+财务结算任务列表属佣金结算，等微店结算数据确认（Q-1017-1/2）后开发。</t>
         </is>
       </c>
     </row>
@@ -5583,8 +5583,8 @@
       </c>
       <c r="H54" s="60" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-缺结算任务详情、商品行占用、预付抵扣和支付凭证。</t>
+          <t xml:space="preserve">10/22 未实现
+结算任务详情与占用明细属佣金结算，等微店结算数据确认（Q-1017-1/2）后开发。</t>
         </is>
       </c>
       <c r="I54" s="52" t="str">
@@ -5611,8 +5611,8 @@
       </c>
       <c r="H55" s="60" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/18 未实现
-缺结算明细、商品行账务流水和入账/付款分别记录。</t>
+          <t xml:space="preserve">10/22 未实现
+结算明细与账务流水属佣金结算，等微店结算数据确认（Q-1017-1/2）后开发。</t>
         </is>
       </c>
       <c r="I55" s="52" t="str">

</xml_diff>